<commit_message>
fix: corrige leitura de codigos PV e alinha processos reais do roteiro com capacidade do APS
</commit_message>
<xml_diff>
--- a/Processos_de_Fabricacao.xlsx
+++ b/Processos_de_Fabricacao.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{429F3660-0FC5-4DF8-988A-EBAF36B6EB1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{423EC461-262D-4769-BFF2-B5092A78593D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Processos" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Processos!$A$1:$X$379</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Processos!$A$1:$X$625</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43562,7 +43562,7 @@
         <v>0</v>
       </c>
       <c r="W578" s="5">
-        <f t="shared" ref="W578:W641" si="9">SUM(C578:V578)</f>
+        <f t="shared" ref="W578:W625" si="9">SUM(C578:V578)</f>
         <v>25</v>
       </c>
     </row>
@@ -46951,7 +46951,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X379" xr:uid="{AF33645A-C41E-42FF-8EC5-04EEB9194698}">
+  <autoFilter ref="A1:X625" xr:uid="{AF33645A-C41E-42FF-8EC5-04EEB9194698}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:W721">
       <sortCondition ref="B1:B379"/>
     </sortState>

</xml_diff>